<commit_message>
final power budget updated
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/power_budget.xlsx
+++ b/docs/05-Power-Budget/power_budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\college\fa25\egr304\individual_datasheet\botilarm.github.io\docs\05-Power-Budget\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8880307E-0CD3-472E-B156-D937D5E400C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A355B2D-1D4E-4BD6-AA6C-9E940E6B2C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="750" yWindow="-120" windowWidth="28170" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -155,9 +155,6 @@
     <t>5V</t>
   </si>
   <si>
-    <t>4797-ZF120A-1205000-ND</t>
-  </si>
-  <si>
     <t>90-264 VAC</t>
   </si>
   <si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>Total Current (mA)</t>
+  </si>
+  <si>
+    <t>ZF120A-1205000</t>
   </si>
 </sst>
 </file>
@@ -258,7 +258,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -267,9 +267,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -380,32 +378,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -413,9 +420,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -515,6 +519,31 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,589 +896,589 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" style="3" customWidth="1"/>
-    <col min="2" max="2" width="45.5" style="3" customWidth="1"/>
-    <col min="3" max="3" width="28.375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="34.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.5" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="13.5" style="3"/>
+    <col min="1" max="1" width="28" style="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="13.5" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
+      <c r="A1" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="46">
         <v>203</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="47">
         <v>1</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
+      <c r="A6" s="48"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="49" t="s">
+      <c r="G7" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="37" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
-      <c r="B8" s="27" t="s">
+      <c r="A8" s="39"/>
+      <c r="B8" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="43">
+      <c r="E8" s="35">
         <v>1</v>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="19">
         <v>500</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="19">
         <f>F8*E8</f>
         <v>500</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="19" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
-      <c r="B9" s="15" t="s">
+      <c r="A9" s="39"/>
+      <c r="B9" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="8">
         <v>1</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="7">
         <v>3000</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="7">
         <f t="shared" ref="G9:G11" si="0">F9*E9</f>
         <v>3000</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
-      <c r="B10" s="15" t="s">
+      <c r="A10" s="39"/>
+      <c r="B10" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="8">
         <v>1</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="10">
         <v>100</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="7">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="47"/>
-      <c r="B11" s="15" t="s">
+    <row r="11" spans="1:8" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="39"/>
+      <c r="B11" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="8">
         <v>1</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="7">
         <v>140</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="7">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-    </row>
-    <row r="13" spans="1:8" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="46" t="s">
+    <row r="12" spans="1:8" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+    </row>
+    <row r="13" spans="1:8" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="45" t="s">
+      <c r="B13" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="45" t="s">
+      <c r="C13" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="49" t="s">
+      <c r="G13" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="G13" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="H13" s="45" t="s">
+      <c r="H13" s="37" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="46"/>
-      <c r="B14" s="27" t="s">
+      <c r="A14" s="38"/>
+      <c r="B14" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="43">
+      <c r="E14" s="35">
         <v>1</v>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="19">
         <v>500</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="19">
         <f t="shared" ref="G14:G17" si="1">E14*F14</f>
         <v>500</v>
       </c>
-      <c r="H14" s="27" t="s">
+      <c r="H14" s="19" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="46"/>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="38"/>
+      <c r="B15" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="8">
         <v>1</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="7">
         <v>3000</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="7">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="46"/>
-      <c r="B16" s="15" t="s">
+      <c r="A16" s="38"/>
+      <c r="B16" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="8">
         <v>1</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="10">
         <v>100</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="7">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="46"/>
-      <c r="B17" s="15" t="s">
+      <c r="A17" s="38"/>
+      <c r="B17" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="8">
         <v>1</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="7">
         <v>140</v>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="7">
         <f t="shared" si="1"/>
         <v>140</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="21" t="s">
+      <c r="A18" s="20"/>
+      <c r="B18" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="15">
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="7">
         <f>SUM(G14:G17)</f>
         <v>3740</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="14" t="s">
+      <c r="A19" s="20"/>
+      <c r="B19" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="19">
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="11">
         <v>0.25</v>
       </c>
-      <c r="H19" s="20"/>
+      <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
-      <c r="B20" s="14" t="s">
+      <c r="A20" s="33"/>
+      <c r="B20" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="15">
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7">
         <f>G18*(1+G19)</f>
         <v>4675</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="24" t="s">
+      <c r="A21" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="8">
         <v>1</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="10">
         <v>5000</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="10">
         <f>E21*F21</f>
         <v>5000</v>
       </c>
-      <c r="H21" s="15" t="s">
+      <c r="H21" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="40"/>
-      <c r="B22" s="38" t="s">
+      <c r="A22" s="32"/>
+      <c r="B22" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="18">
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="10">
         <f>G21-G20</f>
         <v>325</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="H22" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
+      <c r="A23" s="54"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E24" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="E24" s="48" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="G24" s="45" t="s">
+      <c r="B25" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="H24" s="45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="29" t="s">
+      <c r="D25" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="34">
+        <v>5000</v>
+      </c>
+      <c r="G25" s="10">
+        <v>5000</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="42">
+      <c r="B26" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="25">
         <v>5000</v>
       </c>
-      <c r="G25" s="18">
-        <v>5000</v>
-      </c>
-      <c r="H25" s="24" t="s">
+      <c r="G26" s="25">
+        <v>4675</v>
+      </c>
+      <c r="H26" s="26" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="F26" s="33">
-        <v>5000</v>
-      </c>
-      <c r="G26" s="33">
-        <v>4675</v>
-      </c>
-      <c r="H26" s="34" t="s">
-        <v>9</v>
-      </c>
-    </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
-      <c r="B27" s="38" t="s">
+      <c r="A27" s="5"/>
+      <c r="B27" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="35">
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="27">
         <f>G25-G26</f>
         <v>325</v>
       </c>
-      <c r="H27" s="36" t="s">
+      <c r="H27" s="28" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="53" t="s">
+      <c r="A28" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="53"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="53"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="45"/>
+      <c r="H28" s="45"/>
     </row>
     <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="51" t="s">
+      <c r="A29" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="50"/>
-      <c r="C29" s="50"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="50"/>
-      <c r="F29" s="50"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="50"/>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="50"/>
-      <c r="C30" s="50"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>

<commit_message>
comp select power bud everything
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/power_budget.xlsx
+++ b/docs/05-Power-Budget/power_budget.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\college\fa25\egr304\individual_datasheet\botilarm.github.io\docs\05-Power-Budget\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99B620F-5712-48C3-9995-9A2CA5A8714C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A3C2D6-F0F9-49BE-ABE3-1BB8C9142FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="750" yWindow="-120" windowWidth="28170" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="49">
   <si>
     <t>Team Number:</t>
   </si>
@@ -90,15 +90,6 @@
   </si>
   <si>
     <t>Total Remaining Current Available on External Power Source 1</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>External Supply Voltage should be determined by the dropout voltage for highest-voltage regulator (e.g., +14V for a +12V regulator).</t>
-  </si>
-  <si>
-    <t>If you have multiple units in your design (e.g., a base unit and remote unit) then you need a separate power budget for each unit</t>
   </si>
   <si>
     <t>Spark Guard</t>
@@ -238,7 +229,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -247,24 +238,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFEEECE1"/>
         <bgColor rgb="FFEEECE1"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -286,15 +265,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -352,19 +322,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -412,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -422,74 +379,65 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -498,58 +446,47 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,33 +851,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="A1" s="39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="33">
+      <c r="B2" s="30">
         <v>203</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="34" t="s">
-        <v>21</v>
+      <c r="B3" s="31" t="s">
+        <v>18</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="2"/>
@@ -950,11 +887,11 @@
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="34" t="s">
-        <v>22</v>
+      <c r="B4" s="31" t="s">
+        <v>19</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
@@ -964,11 +901,11 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34">
-        <v>1</v>
+      <c r="B5" s="31">
+        <v>2</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="2"/>
@@ -978,8 +915,8 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="35"/>
-      <c r="B6" s="35"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="3"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -988,511 +925,501 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="E7" s="30" t="s">
+      <c r="D7" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="H7" s="30" t="s">
+      <c r="F7" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="27" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="50"/>
-      <c r="B8" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="28">
+      <c r="A8" s="46"/>
+      <c r="B8" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="25">
         <v>1</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="13">
         <v>500</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="13">
         <f>F8*E8</f>
         <v>500</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="50"/>
-      <c r="B9" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="7">
+      <c r="A9" s="46"/>
+      <c r="B9" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="6">
         <v>1</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>3000</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="5">
         <f t="shared" ref="G9:G11" si="0">F9*E9</f>
         <v>3000</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="50"/>
-      <c r="B10" s="38" t="s">
+      <c r="A10" s="46"/>
+      <c r="B10" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="6">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8">
+        <v>0.17</v>
+      </c>
+      <c r="G10" s="5">
+        <f t="shared" si="0"/>
+        <v>0.17</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="46"/>
+      <c r="B11" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E11" s="6">
         <v>1</v>
       </c>
-      <c r="F10" s="9">
-        <v>100</v>
-      </c>
-      <c r="G10" s="6">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="50"/>
-      <c r="B11" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="7">
-        <v>1</v>
-      </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>140</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="5">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-    </row>
-    <row r="13" spans="1:8" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="49" t="s">
+    <row r="12" spans="1:8" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+    </row>
+    <row r="13" spans="1:8" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="30" t="s">
+      <c r="D13" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="30" t="s">
+      <c r="F13" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H13" s="27" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="49"/>
-      <c r="B14" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="28">
+      <c r="A14" s="45"/>
+      <c r="B14" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="25">
         <v>1</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="13">
         <v>500</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="13">
         <f t="shared" ref="G14:G17" si="1">E14*F14</f>
         <v>500</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="49"/>
-      <c r="B15" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="7" t="s">
+      <c r="A15" s="45"/>
+      <c r="B15" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="6">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1500</v>
+      </c>
+      <c r="G15" s="5">
+        <v>1500</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="45"/>
+      <c r="B16" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="7">
+      <c r="D16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6">
         <v>1</v>
       </c>
-      <c r="F15" s="6">
-        <v>1500</v>
-      </c>
-      <c r="G15" s="6">
-        <v>1500</v>
-      </c>
-      <c r="H15" s="6" t="s">
+      <c r="F16" s="8">
+        <v>0.17</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0.17</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="49"/>
-      <c r="B16" s="38" t="s">
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="45"/>
+      <c r="B17" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E17" s="6">
         <v>1</v>
       </c>
-      <c r="F16" s="9">
-        <v>0.4</v>
-      </c>
-      <c r="G16" s="6">
-        <f t="shared" si="1"/>
-        <v>0.4</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="49"/>
-      <c r="B17" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="7">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6">
+      <c r="F17" s="5">
         <v>140</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="5">
         <f t="shared" si="1"/>
         <v>140</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="15"/>
-      <c r="B18" s="45" t="s">
+      <c r="A18" s="14"/>
+      <c r="B18" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="6">
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="5">
         <f>SUM(G14:G17)</f>
-        <v>2140.4</v>
-      </c>
-      <c r="H18" s="6" t="s">
+        <v>2140.17</v>
+      </c>
+      <c r="H18" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="15"/>
-      <c r="B19" s="47" t="s">
+      <c r="A19" s="14"/>
+      <c r="B19" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="10">
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="9">
         <v>0.25</v>
       </c>
-      <c r="H19" s="11"/>
+      <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="26"/>
-      <c r="B20" s="47" t="s">
+      <c r="A20" s="23"/>
+      <c r="B20" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="6">
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="5">
         <f>G18*(1+G19)</f>
-        <v>2675.5</v>
-      </c>
-      <c r="H20" s="6" t="s">
+        <v>2675.2125000000001</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="7">
+      <c r="A21" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="6">
         <v>1</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="8">
         <v>3000</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="8">
         <f>E21*F21</f>
         <v>3000</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="25"/>
-      <c r="B22" s="51" t="s">
+      <c r="A22" s="22"/>
+      <c r="B22" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="9">
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="8">
         <f>G21-G20</f>
-        <v>324.5</v>
-      </c>
-      <c r="H22" s="6" t="s">
+        <v>324.78749999999991</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="40"/>
-      <c r="B23" s="40"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="36" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="E24" s="32" t="s">
+      <c r="E24" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="G24" s="30" t="s">
+      <c r="F24" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H24" s="27" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" s="24">
+        <v>3000</v>
+      </c>
+      <c r="G25" s="8">
+        <v>3000</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="H24" s="30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F25" s="27">
+      <c r="D26" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="19">
         <v>3000</v>
       </c>
-      <c r="G25" s="9">
-        <v>3000</v>
-      </c>
-      <c r="H25" s="13" t="s">
+      <c r="G26" s="19">
+        <f>G20</f>
+        <v>2675.2125000000001</v>
+      </c>
+      <c r="H26" s="20" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="41" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="20">
-        <v>3000</v>
-      </c>
-      <c r="G26" s="20">
-        <f>G20</f>
-        <v>2675.5</v>
-      </c>
-      <c r="H26" s="21" t="s">
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="50"/>
+      <c r="B27" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="8">
+        <f>G25-G26</f>
+        <v>324.78749999999991</v>
+      </c>
+      <c r="H27" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="22">
-        <f>G25-G26</f>
-        <v>324.5</v>
-      </c>
-      <c r="H27" s="23" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="53"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="53"/>
-    </row>
-    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="54" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-    </row>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="56" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28"/>
+      <c r="B28"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29"/>
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="H29"/>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30"/>
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="15"/>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="8">
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A30:H30"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B18:F18"/>

</xml_diff>